<commit_message>
Isolate CodeRabbit review scope source changes
</commit_message>
<xml_diff>
--- a/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
+++ b/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wbowe\OneDrive\Desktop\project\DMIS_UpdatedVersion\docs\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F17D9C9-D9CF-4FF3-81BF-2E3715E7D989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3830B1A-8FB9-4F76-A922-045469650ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -4277,17 +4277,17 @@
     <xf numFmtId="0" fontId="12" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -4621,7 +4621,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="43"/>
@@ -4634,7 +4634,7 @@
       <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="43"/>
@@ -5191,7 +5191,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>637</v>
       </c>
       <c r="B1" s="43"/>
@@ -5206,7 +5206,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>638</v>
       </c>
       <c r="B2" s="43"/>
@@ -5221,7 +5221,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>639</v>
       </c>
       <c r="B3" s="43"/>
@@ -5566,7 +5566,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>663</v>
       </c>
       <c r="B1" s="43"/>
@@ -5581,7 +5581,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>664</v>
       </c>
       <c r="B2" s="43"/>
@@ -5596,7 +5596,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>665</v>
       </c>
       <c r="B3" s="43"/>
@@ -6493,7 +6493,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>732</v>
       </c>
       <c r="B1" s="43"/>
@@ -6508,7 +6508,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>733</v>
       </c>
       <c r="B2" s="43"/>
@@ -6523,7 +6523,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>734</v>
       </c>
       <c r="B3" s="43"/>
@@ -6574,19 +6574,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="46" t="s">
         <v>735</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="47"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -6821,19 +6821,19 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="46" t="s">
         <v>752</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
-      <c r="K15" s="47"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="48"/>
     </row>
     <row r="16" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
@@ -7012,19 +7012,19 @@
       <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="46" t="s">
         <v>765</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="47"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="48"/>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
@@ -7274,7 +7274,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>780</v>
       </c>
       <c r="B1" s="43"/>
@@ -7289,7 +7289,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>781</v>
       </c>
       <c r="B2" s="43"/>
@@ -7304,7 +7304,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>782</v>
       </c>
       <c r="B3" s="43"/>
@@ -7620,7 +7620,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>802</v>
       </c>
       <c r="B1" s="43"/>
@@ -7635,7 +7635,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>803</v>
       </c>
       <c r="B2" s="43"/>
@@ -7650,7 +7650,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>804</v>
       </c>
       <c r="B3" s="43"/>
@@ -8262,7 +8262,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>850</v>
       </c>
       <c r="B1" s="43"/>
@@ -8277,7 +8277,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>851</v>
       </c>
       <c r="B2" s="43"/>
@@ -8292,7 +8292,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>852</v>
       </c>
       <c r="B3" s="43"/>
@@ -8933,7 +8933,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>900</v>
       </c>
       <c r="B1" s="43"/>
@@ -8948,7 +8948,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>901</v>
       </c>
       <c r="B2" s="43"/>
@@ -8963,7 +8963,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>902</v>
       </c>
       <c r="B3" s="43"/>
@@ -9013,7 +9013,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>903</v>
       </c>
@@ -9042,7 +9042,7 @@
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
         <v>908</v>
       </c>
@@ -9104,7 +9104,7 @@
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
     </row>
-    <row r="9" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="98.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
         <v>912</v>
       </c>
@@ -9135,7 +9135,7 @@
       <c r="J9" s="18"/>
       <c r="K9" s="18"/>
     </row>
-    <row r="10" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
         <v>915</v>
       </c>
@@ -11166,7 +11166,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>81</v>
       </c>
       <c r="B1" s="43"/>
@@ -11181,7 +11181,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="43"/>
@@ -11196,7 +11196,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>83</v>
       </c>
       <c r="B3" s="43"/>
@@ -11247,19 +11247,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="47"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -11730,19 +11730,19 @@
       <c r="K22" s="4"/>
     </row>
     <row r="23" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="46" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
-      <c r="K23" s="47"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="48"/>
     </row>
     <row r="24" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
@@ -12151,19 +12151,19 @@
       <c r="K37" s="18"/>
     </row>
     <row r="38" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="45" t="s">
+      <c r="A38" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
-      <c r="K38" s="47"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="47"/>
+      <c r="F38" s="47"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="47"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="47"/>
+      <c r="K38" s="48"/>
     </row>
     <row r="39" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="23" t="s">
@@ -12197,19 +12197,19 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="45" t="s">
+      <c r="A40" s="46" t="s">
         <v>135</v>
       </c>
-      <c r="B40" s="46"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="46"/>
-      <c r="F40" s="46"/>
-      <c r="G40" s="46"/>
-      <c r="H40" s="46"/>
-      <c r="I40" s="46"/>
-      <c r="J40" s="46"/>
-      <c r="K40" s="47"/>
+      <c r="B40" s="47"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="47"/>
+      <c r="J40" s="47"/>
+      <c r="K40" s="48"/>
     </row>
     <row r="41" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="23" t="s">
@@ -12277,13 +12277,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A40:K40"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A23:K23"/>
     <mergeCell ref="A6:K6"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A38:K38"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A40:K40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12907,16 +12907,16 @@
       <c r="A4" s="53" t="s">
         <v>1270</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="47"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="48"/>
     </row>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39" t="s">
@@ -12989,11 +12989,11 @@
       <c r="A8" s="53" t="s">
         <v>1278</v>
       </c>
-      <c r="B8" s="46"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="47"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="48"/>
     </row>
     <row r="9" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="39" t="s">
@@ -13082,7 +13082,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>172</v>
       </c>
       <c r="B1" s="43"/>
@@ -13097,7 +13097,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>173</v>
       </c>
       <c r="B2" s="43"/>
@@ -13112,7 +13112,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>174</v>
       </c>
       <c r="B3" s="43"/>
@@ -13163,19 +13163,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="47"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="48"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -13296,19 +13296,19 @@
       <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="46" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="47"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="48"/>
     </row>
     <row r="12" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
@@ -13847,19 +13847,19 @@
       <c r="K29" s="18"/>
     </row>
     <row r="30" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="46" t="s">
         <v>224</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="47"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="47"/>
+      <c r="D30" s="47"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="48"/>
     </row>
     <row r="31" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
@@ -14067,19 +14067,19 @@
       <c r="K37" s="18"/>
     </row>
     <row r="38" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="45" t="s">
+      <c r="A38" s="46" t="s">
         <v>238</v>
       </c>
-      <c r="B38" s="46"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
-      <c r="K38" s="47"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="47"/>
+      <c r="F38" s="47"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="47"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="47"/>
+      <c r="K38" s="48"/>
     </row>
     <row r="39" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
@@ -14229,19 +14229,19 @@
       <c r="K43" s="18"/>
     </row>
     <row r="44" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="45" t="s">
+      <c r="A44" s="46" t="s">
         <v>250</v>
       </c>
-      <c r="B44" s="46"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="46"/>
-      <c r="E44" s="46"/>
-      <c r="F44" s="46"/>
-      <c r="G44" s="46"/>
-      <c r="H44" s="46"/>
-      <c r="I44" s="46"/>
-      <c r="J44" s="46"/>
-      <c r="K44" s="47"/>
+      <c r="B44" s="47"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="47"/>
+      <c r="E44" s="47"/>
+      <c r="F44" s="47"/>
+      <c r="G44" s="47"/>
+      <c r="H44" s="47"/>
+      <c r="I44" s="47"/>
+      <c r="J44" s="47"/>
+      <c r="K44" s="48"/>
     </row>
     <row r="45" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
@@ -14395,19 +14395,19 @@
       <c r="K49" s="18"/>
     </row>
     <row r="50" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="45" t="s">
+      <c r="A50" s="46" t="s">
         <v>261</v>
       </c>
-      <c r="B50" s="46"/>
-      <c r="C50" s="46"/>
-      <c r="D50" s="46"/>
-      <c r="E50" s="46"/>
-      <c r="F50" s="46"/>
-      <c r="G50" s="46"/>
-      <c r="H50" s="46"/>
-      <c r="I50" s="46"/>
-      <c r="J50" s="46"/>
-      <c r="K50" s="47"/>
+      <c r="B50" s="47"/>
+      <c r="C50" s="47"/>
+      <c r="D50" s="47"/>
+      <c r="E50" s="47"/>
+      <c r="F50" s="47"/>
+      <c r="G50" s="47"/>
+      <c r="H50" s="47"/>
+      <c r="I50" s="47"/>
+      <c r="J50" s="47"/>
+      <c r="K50" s="48"/>
     </row>
     <row r="51" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
@@ -14646,19 +14646,19 @@
       <c r="K58" s="4"/>
     </row>
     <row r="59" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="45" t="s">
+      <c r="A59" s="46" t="s">
         <v>278</v>
       </c>
-      <c r="B59" s="46"/>
-      <c r="C59" s="46"/>
-      <c r="D59" s="46"/>
-      <c r="E59" s="46"/>
-      <c r="F59" s="46"/>
-      <c r="G59" s="46"/>
-      <c r="H59" s="46"/>
-      <c r="I59" s="46"/>
-      <c r="J59" s="46"/>
-      <c r="K59" s="47"/>
+      <c r="B59" s="47"/>
+      <c r="C59" s="47"/>
+      <c r="D59" s="47"/>
+      <c r="E59" s="47"/>
+      <c r="F59" s="47"/>
+      <c r="G59" s="47"/>
+      <c r="H59" s="47"/>
+      <c r="I59" s="47"/>
+      <c r="J59" s="47"/>
+      <c r="K59" s="48"/>
     </row>
     <row r="60" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="21" t="s">
@@ -14922,19 +14922,19 @@
       <c r="K68" s="4"/>
     </row>
     <row r="69" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="45" t="s">
+      <c r="A69" s="46" t="s">
         <v>297</v>
       </c>
-      <c r="B69" s="46"/>
-      <c r="C69" s="46"/>
-      <c r="D69" s="46"/>
-      <c r="E69" s="46"/>
-      <c r="F69" s="46"/>
-      <c r="G69" s="46"/>
-      <c r="H69" s="46"/>
-      <c r="I69" s="46"/>
-      <c r="J69" s="46"/>
-      <c r="K69" s="47"/>
+      <c r="B69" s="47"/>
+      <c r="C69" s="47"/>
+      <c r="D69" s="47"/>
+      <c r="E69" s="47"/>
+      <c r="F69" s="47"/>
+      <c r="G69" s="47"/>
+      <c r="H69" s="47"/>
+      <c r="I69" s="47"/>
+      <c r="J69" s="47"/>
+      <c r="K69" s="48"/>
     </row>
     <row r="70" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="21" t="s">
@@ -15206,19 +15206,19 @@
       <c r="K78" s="4"/>
     </row>
     <row r="79" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="45" t="s">
+      <c r="A79" s="46" t="s">
         <v>316</v>
       </c>
-      <c r="B79" s="46"/>
-      <c r="C79" s="46"/>
-      <c r="D79" s="46"/>
-      <c r="E79" s="46"/>
-      <c r="F79" s="46"/>
-      <c r="G79" s="46"/>
-      <c r="H79" s="46"/>
-      <c r="I79" s="46"/>
-      <c r="J79" s="46"/>
-      <c r="K79" s="47"/>
+      <c r="B79" s="47"/>
+      <c r="C79" s="47"/>
+      <c r="D79" s="47"/>
+      <c r="E79" s="47"/>
+      <c r="F79" s="47"/>
+      <c r="G79" s="47"/>
+      <c r="H79" s="47"/>
+      <c r="I79" s="47"/>
+      <c r="J79" s="47"/>
+      <c r="K79" s="48"/>
     </row>
     <row r="80" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="21" t="s">
@@ -15401,19 +15401,19 @@
       <c r="K85" s="18"/>
     </row>
     <row r="86" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="45" t="s">
+      <c r="A86" s="46" t="s">
         <v>329</v>
       </c>
-      <c r="B86" s="46"/>
-      <c r="C86" s="46"/>
-      <c r="D86" s="46"/>
-      <c r="E86" s="46"/>
-      <c r="F86" s="46"/>
-      <c r="G86" s="46"/>
-      <c r="H86" s="46"/>
-      <c r="I86" s="46"/>
-      <c r="J86" s="46"/>
-      <c r="K86" s="47"/>
+      <c r="B86" s="47"/>
+      <c r="C86" s="47"/>
+      <c r="D86" s="47"/>
+      <c r="E86" s="47"/>
+      <c r="F86" s="47"/>
+      <c r="G86" s="47"/>
+      <c r="H86" s="47"/>
+      <c r="I86" s="47"/>
+      <c r="J86" s="47"/>
+      <c r="K86" s="48"/>
     </row>
     <row r="87" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="17" t="s">
@@ -15687,19 +15687,19 @@
       <c r="K95" s="18"/>
     </row>
     <row r="96" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="45" t="s">
+      <c r="A96" s="46" t="s">
         <v>348</v>
       </c>
-      <c r="B96" s="46"/>
-      <c r="C96" s="46"/>
-      <c r="D96" s="46"/>
-      <c r="E96" s="46"/>
-      <c r="F96" s="46"/>
-      <c r="G96" s="46"/>
-      <c r="H96" s="46"/>
-      <c r="I96" s="46"/>
-      <c r="J96" s="46"/>
-      <c r="K96" s="47"/>
+      <c r="B96" s="47"/>
+      <c r="C96" s="47"/>
+      <c r="D96" s="47"/>
+      <c r="E96" s="47"/>
+      <c r="F96" s="47"/>
+      <c r="G96" s="47"/>
+      <c r="H96" s="47"/>
+      <c r="I96" s="47"/>
+      <c r="J96" s="47"/>
+      <c r="K96" s="48"/>
     </row>
     <row r="97" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="17" t="s">
@@ -15789,19 +15789,19 @@
       <c r="K99" s="18"/>
     </row>
     <row r="100" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="45" t="s">
+      <c r="A100" s="46" t="s">
         <v>224</v>
       </c>
-      <c r="B100" s="46"/>
-      <c r="C100" s="46"/>
-      <c r="D100" s="46"/>
-      <c r="E100" s="46"/>
-      <c r="F100" s="46"/>
-      <c r="G100" s="46"/>
-      <c r="H100" s="46"/>
-      <c r="I100" s="46"/>
-      <c r="J100" s="46"/>
-      <c r="K100" s="47"/>
+      <c r="B100" s="47"/>
+      <c r="C100" s="47"/>
+      <c r="D100" s="47"/>
+      <c r="E100" s="47"/>
+      <c r="F100" s="47"/>
+      <c r="G100" s="47"/>
+      <c r="H100" s="47"/>
+      <c r="I100" s="47"/>
+      <c r="J100" s="47"/>
+      <c r="K100" s="48"/>
     </row>
     <row r="101" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="23" t="s">
@@ -15906,6 +15906,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A100:K100"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A96:K96"/>
+    <mergeCell ref="A86:K86"/>
+    <mergeCell ref="A59:K59"/>
+    <mergeCell ref="A38:K38"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A44:K44"/>
@@ -15914,13 +15921,6 @@
     <mergeCell ref="A6:K6"/>
     <mergeCell ref="A69:K69"/>
     <mergeCell ref="A50:K50"/>
-    <mergeCell ref="A100:K100"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="A96:K96"/>
-    <mergeCell ref="A86:K86"/>
-    <mergeCell ref="A59:K59"/>
-    <mergeCell ref="A38:K38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15948,7 +15948,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>359</v>
       </c>
       <c r="B1" s="43"/>
@@ -15963,7 +15963,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>360</v>
       </c>
       <c r="B2" s="43"/>
@@ -15978,7 +15978,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>361</v>
       </c>
       <c r="B3" s="43"/>
@@ -16704,7 +16704,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>417</v>
       </c>
       <c r="B1" s="43"/>
@@ -16719,7 +16719,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>418</v>
       </c>
       <c r="B2" s="43"/>
@@ -16734,7 +16734,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>419</v>
       </c>
       <c r="B3" s="43"/>
@@ -17257,7 +17257,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>460</v>
       </c>
       <c r="B1" s="43"/>
@@ -17272,7 +17272,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>461</v>
       </c>
       <c r="B2" s="43"/>
@@ -17287,7 +17287,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>462</v>
       </c>
       <c r="B3" s="43"/>
@@ -17990,7 +17990,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>516</v>
       </c>
       <c r="B1" s="43"/>
@@ -18005,7 +18005,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>517</v>
       </c>
       <c r="B2" s="43"/>
@@ -18020,7 +18020,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>518</v>
       </c>
       <c r="B3" s="43"/>
@@ -18667,7 +18667,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>567</v>
       </c>
       <c r="B1" s="43"/>
@@ -18682,7 +18682,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>568</v>
       </c>
       <c r="B2" s="43"/>
@@ -18697,7 +18697,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>569</v>
       </c>
       <c r="B3" s="43"/>
@@ -19108,7 +19108,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>601</v>
       </c>
       <c r="B1" s="43"/>
@@ -19123,7 +19123,7 @@
       <c r="K1" s="43"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="42" t="s">
         <v>602</v>
       </c>
       <c r="B2" s="43"/>
@@ -19138,7 +19138,7 @@
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="45" t="s">
         <v>603</v>
       </c>
       <c r="B3" s="43"/>

</xml_diff>

<commit_message>
Align requirements design guidance with backlog v3.2
</commit_message>
<xml_diff>
--- a/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
+++ b/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wbowe\OneDrive\Desktop\project\DMIS_UpdatedVersion\docs\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3830B1A-8FB9-4F76-A922-045469650ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0E0B07-9AEB-4FBA-B3C9-7B2CF446201D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3717" uniqueCount="1283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3736" uniqueCount="1289">
   <si>
     <t>DMIS Product Backlog v3.2 — Aligned to Requirements Specification v6.1 (Cleaned)</t>
   </si>
@@ -3903,6 +3903,24 @@
   </si>
   <si>
     <t>INSTRUCTIONS: When the governance board approves an item, update its status to APPROVED, record the approval date, then move the row to the appropriate EP or BR sheet and update the Summary totals. Do not develop, test, or deploy any item from this sheet while status shows NOT APPROVED.</t>
+  </si>
+  <si>
+    <t>FR10.29</t>
+  </si>
+  <si>
+    <t>Digital Signature</t>
+  </si>
+  <si>
+    <t>The system shall support digital signature capture, allowing beneficiaries or relief requesters to electronically sign waybills, goods-received notes, and other distribution forms to acknowledge receipt of goods.</t>
+  </si>
+  <si>
+    <t>v6.1</t>
+  </si>
+  <si>
+    <t>FR10.30</t>
+  </si>
+  <si>
+    <t>The system shall consume imported donation and relief shipment data from Jamaica Customs' ASYCUDA system via an approved API or data feed, capturing Port of Entry clearance status, consignment details, and donor/item classification for all goods entering through designated ports. Ingested records shall be matched to corresponding donation records within DMIS, with source attribution and freshness indicators displayed on relevant dashboards.</t>
   </si>
 </sst>
 </file>
@@ -4603,6 +4621,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D18A0413-D404-4D98-AC46-064FAB80DEC5}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;bad4e2ad-6687-437d-8f6d-313fe9509767&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
@@ -5549,7 +5589,7 @@
   <sheetPr>
     <tabColor rgb="FF2C5F8A"/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6399,7 +6439,7 @@
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
     </row>
-    <row r="31" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
         <v>728</v>
       </c>
@@ -6460,6 +6500,70 @@
       </c>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
+    </row>
+    <row r="33" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="21" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1284</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4" t="s">
+        <v>1286</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="K33" s="4"/>
+    </row>
+    <row r="34" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="21" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>682</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>1286</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="K34" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -15906,13 +16010,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A100:K100"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="A96:K96"/>
-    <mergeCell ref="A86:K86"/>
-    <mergeCell ref="A59:K59"/>
-    <mergeCell ref="A38:K38"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A44:K44"/>
@@ -15921,6 +16018,13 @@
     <mergeCell ref="A6:K6"/>
     <mergeCell ref="A69:K69"/>
     <mergeCell ref="A50:K50"/>
+    <mergeCell ref="A100:K100"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A96:K96"/>
+    <mergeCell ref="A86:K86"/>
+    <mergeCell ref="A59:K59"/>
+    <mergeCell ref="A38:K38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Align needs list workflow persistence
</commit_message>
<xml_diff>
--- a/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
+++ b/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wbowe\OneDrive\Desktop\project\DMIS_UpdatedVersion\docs\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E72714E7-224E-40FC-B40C-624F48989D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9365B87E-5D26-46A2-B901-76766CDA2E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update operations queues and backlog asset
</commit_message>
<xml_diff>
--- a/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
+++ b/docs/attached_assets/DMIS_Product_Backlog_v3.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wbowe\OneDrive\Desktop\project\DMIS_UpdatedVersion\docs\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883815CB-CE7F-4CC2-A368-B43EB3C0C8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369FDDAD-7F6C-41EE-8337-A78104D5533A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4543" uniqueCount="1556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4596" uniqueCount="1575">
   <si>
     <t>DMIS Product Backlog v3.2 — Aligned to Requirements Specification v6.1 (Cleaned)</t>
   </si>
@@ -4735,13 +4735,70 @@
   </si>
   <si>
     <t>FR-CON-36G</t>
+  </si>
+  <si>
+    <t>FR02.99</t>
+  </si>
+  <si>
+    <t>The system shall treat ODPEM HQ/NATIONAL tenant needs lists as replenishment sourcing records only. ODPEM HQ needs lists shall execute through approved transfers, donation allocation/export/broadcast, procurement recommendations, or procurement records. ODPEM HQ needs-list demand shall not be converted into an ODPEM-owned relief request for ODPEM HQ stock needs.</t>
+  </si>
+  <si>
+    <t>Request Authority Discipline</t>
+  </si>
+  <si>
+    <t>Relief Request Authority</t>
+  </si>
+  <si>
+    <t>The system shall allow relief requests to be created only by authorized requester tenants, including parish councils, shelters, direct operational tenants, or approved parent/request-authority tenants acting for entities under their control. ODPEM HQ/NATIONAL users shall not create relief requests for ODPEM HQ needs-list demand.</t>
+  </si>
+  <si>
+    <t>ODPEM Transitional Intake Bridge</t>
+  </si>
+  <si>
+    <t>ODPEM HQ authorized bridge users shall be able to create relief requests on behalf of shelters, parish councils, or other approved requester entities only as a transitional intake channel for phone, email, or other off-platform requests. The request owner/beneficiary context shall remain the represented requester entity, and the system shall retain the on-behalf origin for audit.</t>
+  </si>
+  <si>
+    <t>FR13.19</t>
+  </si>
+  <si>
+    <t>Request Authority &amp; Participation Model</t>
+  </si>
+  <si>
+    <t>Tenant participation configuration shall distinguish direct requester tenants, parent/request-authority tenants, subordinate entities, ODPEM HQ national bridge users, and ODPEM HQ replenishment-only activity. NATIONAL/ODPEM tenancy may maintain replenishment needs lists and create on-behalf relief requests for approved external requesters, but shall not self-request relief against its own needs-list demand.</t>
+  </si>
+  <si>
+    <t>ODPEM HQ/NATIONAL needs lists are replenishment demand records for stock readiness and shall be fulfilled through approved transfers, donation sourcing, or procurement. They shall not generate ODPEM-owned relief requests for ODPEM HQ stock needs.</t>
+  </si>
+  <si>
+    <t>EP-02, EP-05, EP-13</t>
+  </si>
+  <si>
+    <t>BR01.32</t>
+  </si>
+  <si>
+    <t>A relief request created by ODPEM HQ on behalf of an off-platform requester shall retain the represented requester/beneficiary ownership, record the ODPEM bridge origin, and remain auditable as transitional intake rather than ODPEM self-service demand.</t>
+  </si>
+  <si>
+    <t>EP-05, EP-13</t>
+  </si>
+  <si>
+    <t>Needs-list ownership and relief-request ownership shall not be conflated. ODPEM HQ may replenish stock and bridge external/off-platform requests, but must not create ODPEM-owned relief requests for ODPEM HQ needs-list demand.</t>
+  </si>
+  <si>
+    <t>FR05.78</t>
+  </si>
+  <si>
+    <t>FR05.79</t>
+  </si>
+  <si>
+    <t>BR01.33</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4850,6 +4907,13 @@
     <font>
       <sz val="9"/>
       <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1A7A3A"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -5082,7 +5146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -5306,16 +5370,9 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -5332,63 +5389,16 @@
     <xf numFmtId="0" fontId="5" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5421,9 +5431,113 @@
     <xf numFmtId="0" fontId="18" fillId="21" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5764,30 +5878,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
     </row>
     <row r="2" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
     </row>
     <row r="3" spans="1:9" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6315,7 +6429,7 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="89" t="s">
+      <c r="A32" s="86" t="s">
         <v>1476</v>
       </c>
     </row>
@@ -6350,49 +6464,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>633</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>634</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>635</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6725,49 +6839,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>659</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>660</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>661</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -7788,7 +7902,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="58.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="91" t="s">
+      <c r="A38" s="88" t="s">
         <v>1459</v>
       </c>
       <c r="B38" s="60" t="s">
@@ -7818,7 +7932,7 @@
       <c r="J38" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="K38" s="92"/>
+      <c r="K38" s="89"/>
     </row>
     <row r="39" spans="1:11" ht="85.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="74" t="s">
@@ -7851,10 +7965,10 @@
       <c r="J39" s="65" t="s">
         <v>166</v>
       </c>
-      <c r="K39" s="93"/>
+      <c r="K39" s="90"/>
     </row>
     <row r="40" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="91" t="s">
+      <c r="A40" s="88" t="s">
         <v>1462</v>
       </c>
       <c r="B40" s="60" t="s">
@@ -7884,7 +7998,7 @@
       <c r="J40" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="K40" s="92"/>
+      <c r="K40" s="89"/>
     </row>
     <row r="41" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A41" s="73" t="s">
@@ -7950,49 +8064,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>728</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>729</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>730</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -8031,19 +8145,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="99" t="s">
+      <c r="A6" s="113" t="s">
         <v>731</v>
       </c>
-      <c r="B6" s="100"/>
-      <c r="C6" s="100"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="101"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="114"/>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="114"/>
+      <c r="J6" s="114"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -8278,19 +8392,19 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="99" t="s">
+      <c r="A15" s="113" t="s">
         <v>748</v>
       </c>
-      <c r="B15" s="100"/>
-      <c r="C15" s="100"/>
-      <c r="D15" s="100"/>
-      <c r="E15" s="100"/>
-      <c r="F15" s="100"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="100"/>
-      <c r="I15" s="100"/>
-      <c r="J15" s="100"/>
-      <c r="K15" s="101"/>
+      <c r="B15" s="114"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="114"/>
+      <c r="E15" s="114"/>
+      <c r="F15" s="114"/>
+      <c r="G15" s="114"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="114"/>
+      <c r="J15" s="114"/>
+      <c r="K15" s="115"/>
     </row>
     <row r="16" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
@@ -8469,19 +8583,19 @@
       <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="99" t="s">
+      <c r="A22" s="113" t="s">
         <v>761</v>
       </c>
-      <c r="B22" s="100"/>
-      <c r="C22" s="100"/>
-      <c r="D22" s="100"/>
-      <c r="E22" s="100"/>
-      <c r="F22" s="100"/>
-      <c r="G22" s="100"/>
-      <c r="H22" s="100"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="100"/>
-      <c r="K22" s="101"/>
+      <c r="B22" s="114"/>
+      <c r="C22" s="114"/>
+      <c r="D22" s="114"/>
+      <c r="E22" s="114"/>
+      <c r="F22" s="114"/>
+      <c r="G22" s="114"/>
+      <c r="H22" s="114"/>
+      <c r="I22" s="114"/>
+      <c r="J22" s="114"/>
+      <c r="K22" s="115"/>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
@@ -8731,49 +8845,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>776</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>777</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>778</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -9060,7 +9174,7 @@
   <sheetPr>
     <tabColor rgb="FF2C5F8A"/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -9077,49 +9191,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>798</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>799</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>800</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -9451,7 +9565,7 @@
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
     </row>
-    <row r="16" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>828</v>
       </c>
@@ -9480,7 +9594,7 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
         <v>830</v>
       </c>
@@ -9659,33 +9773,66 @@
       <c r="K22" s="4"/>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="69" t="s">
         <v>843</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="70" t="s">
         <v>844</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="71" t="s">
         <v>845</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="72" t="s">
         <v>122</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="18" t="s">
+      <c r="E23" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="70" t="s">
         <v>665</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="70" t="s">
         <v>640</v>
       </c>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="70" t="s">
+        <v>100</v>
+      </c>
+      <c r="J23" s="70"/>
+      <c r="K23" s="70"/>
+    </row>
+    <row r="24" spans="1:11" ht="68.400000000000006" x14ac:dyDescent="0.3">
+      <c r="A24" s="126" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B24" s="127" t="s">
+        <v>1564</v>
+      </c>
+      <c r="C24" s="128" t="s">
+        <v>1565</v>
+      </c>
+      <c r="D24" s="127" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24" s="127" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" s="127" t="s">
+        <v>665</v>
+      </c>
+      <c r="G24" s="127" t="s">
+        <v>640</v>
+      </c>
+      <c r="H24" s="127" t="s">
+        <v>1558</v>
+      </c>
+      <c r="I24" s="138" t="s">
+        <v>1453</v>
+      </c>
+      <c r="J24" s="138" t="s">
+        <v>166</v>
+      </c>
+      <c r="K24" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -9719,49 +9866,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>847</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>848</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -10390,49 +10537,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>896</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>897</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>898</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -11157,20 +11304,20 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="2" max="2" width="65" style="51" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="116" t="s">
         <v>952</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
     </row>
     <row r="2" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -11632,10 +11779,10 @@
       <c r="A32" s="82" t="s">
         <v>1021</v>
       </c>
-      <c r="B32" s="85" t="s">
+      <c r="B32" s="83" t="s">
         <v>1022</v>
       </c>
-      <c r="C32" s="87" t="s">
+      <c r="C32" s="84" t="s">
         <v>1020</v>
       </c>
       <c r="D32" s="82" t="s">
@@ -11645,36 +11792,56 @@
         <v>166</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="83" t="s">
+    <row r="33" spans="1:5" ht="58.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="139" t="s">
         <v>1276</v>
       </c>
-      <c r="B33" s="86" t="s">
+      <c r="B33" s="145" t="s">
         <v>1451</v>
       </c>
-      <c r="C33" s="88" t="s">
+      <c r="C33" s="123" t="s">
         <v>1452</v>
       </c>
-      <c r="D33" s="83" t="s">
+      <c r="D33" s="139" t="s">
         <v>1453</v>
       </c>
-      <c r="E33" s="84" t="s">
+      <c r="E33" s="140" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="38"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="38"/>
+    <row r="34" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="139" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B34" s="145" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C34" s="123" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D34" s="139" t="s">
+        <v>1453</v>
+      </c>
+      <c r="E34" s="140" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="35" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="38"/>
-      <c r="B35" s="38"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="38"/>
+      <c r="A35" s="133" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B35" s="132" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C35" s="85" t="s">
+        <v>1570</v>
+      </c>
+      <c r="D35" s="133" t="s">
+        <v>1453</v>
+      </c>
+      <c r="E35" s="141" t="s">
+        <v>166</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11699,12 +11866,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="116" t="s">
         <v>1023</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -12223,16 +12390,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="116" t="s">
         <v>1103</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
     </row>
     <row r="2" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -12633,49 +12800,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -12714,19 +12881,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="99" t="s">
+      <c r="A6" s="113" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="100"/>
-      <c r="C6" s="100"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="101"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="114"/>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="114"/>
+      <c r="J6" s="114"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -13197,19 +13364,19 @@
       <c r="K22" s="4"/>
     </row>
     <row r="23" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="99" t="s">
+      <c r="A23" s="113" t="s">
         <v>134</v>
       </c>
-      <c r="B23" s="100"/>
-      <c r="C23" s="100"/>
-      <c r="D23" s="100"/>
-      <c r="E23" s="100"/>
-      <c r="F23" s="100"/>
-      <c r="G23" s="100"/>
-      <c r="H23" s="100"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="100"/>
-      <c r="K23" s="101"/>
+      <c r="B23" s="114"/>
+      <c r="C23" s="114"/>
+      <c r="D23" s="114"/>
+      <c r="E23" s="114"/>
+      <c r="F23" s="114"/>
+      <c r="G23" s="114"/>
+      <c r="H23" s="114"/>
+      <c r="I23" s="114"/>
+      <c r="J23" s="114"/>
+      <c r="K23" s="115"/>
     </row>
     <row r="24" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
@@ -13618,19 +13785,19 @@
       <c r="K37" s="18"/>
     </row>
     <row r="38" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="99" t="s">
+      <c r="A38" s="113" t="s">
         <v>94</v>
       </c>
-      <c r="B38" s="100"/>
-      <c r="C38" s="100"/>
-      <c r="D38" s="100"/>
-      <c r="E38" s="100"/>
-      <c r="F38" s="100"/>
-      <c r="G38" s="100"/>
-      <c r="H38" s="100"/>
-      <c r="I38" s="100"/>
-      <c r="J38" s="100"/>
-      <c r="K38" s="101"/>
+      <c r="B38" s="114"/>
+      <c r="C38" s="114"/>
+      <c r="D38" s="114"/>
+      <c r="E38" s="114"/>
+      <c r="F38" s="114"/>
+      <c r="G38" s="114"/>
+      <c r="H38" s="114"/>
+      <c r="I38" s="114"/>
+      <c r="J38" s="114"/>
+      <c r="K38" s="115"/>
     </row>
     <row r="39" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="23" t="s">
@@ -13664,19 +13831,19 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="99" t="s">
+      <c r="A40" s="113" t="s">
         <v>134</v>
       </c>
-      <c r="B40" s="100"/>
-      <c r="C40" s="100"/>
-      <c r="D40" s="100"/>
-      <c r="E40" s="100"/>
-      <c r="F40" s="100"/>
-      <c r="G40" s="100"/>
-      <c r="H40" s="100"/>
-      <c r="I40" s="100"/>
-      <c r="J40" s="100"/>
-      <c r="K40" s="101"/>
+      <c r="B40" s="114"/>
+      <c r="C40" s="114"/>
+      <c r="D40" s="114"/>
+      <c r="E40" s="114"/>
+      <c r="F40" s="114"/>
+      <c r="G40" s="114"/>
+      <c r="H40" s="114"/>
+      <c r="I40" s="114"/>
+      <c r="J40" s="114"/>
+      <c r="K40" s="115"/>
     </row>
     <row r="41" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="23" t="s">
@@ -13773,15 +13940,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="116" t="s">
         <v>1177</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
     </row>
     <row r="2" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -14051,7 +14218,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -14060,11 +14227,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="117" t="s">
         <v>1220</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -14155,13 +14322,24 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="129" t="s">
         <v>1237</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="130" t="s">
         <v>1238</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="130" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A11" s="142" t="s">
+        <v>1558</v>
+      </c>
+      <c r="B11" s="143" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C11" s="144" t="s">
         <v>1225</v>
       </c>
     </row>
@@ -14190,14 +14368,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="118" t="s">
         <v>1239</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="34" t="s">
@@ -14340,50 +14518,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="122" t="s">
         <v>1264</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="52.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="107" t="s">
+      <c r="A2" s="121" t="s">
         <v>1265</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="106" t="s">
+      <c r="A4" s="120" t="s">
         <v>1266</v>
       </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
-      <c r="D4" s="100"/>
-      <c r="E4" s="100"/>
-      <c r="F4" s="100"/>
-      <c r="G4" s="100"/>
-      <c r="H4" s="100"/>
-      <c r="I4" s="100"/>
-      <c r="J4" s="100"/>
-      <c r="K4" s="101"/>
+      <c r="B4" s="114"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="114"/>
+      <c r="E4" s="114"/>
+      <c r="F4" s="114"/>
+      <c r="G4" s="114"/>
+      <c r="H4" s="114"/>
+      <c r="I4" s="114"/>
+      <c r="J4" s="114"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39" t="s">
@@ -14453,14 +14631,14 @@
     </row>
     <row r="7" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="106" t="s">
+      <c r="A8" s="120" t="s">
         <v>1274</v>
       </c>
-      <c r="B8" s="100"/>
-      <c r="C8" s="100"/>
-      <c r="D8" s="100"/>
-      <c r="E8" s="100"/>
-      <c r="F8" s="101"/>
+      <c r="B8" s="114"/>
+      <c r="C8" s="114"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
+      <c r="F8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="39" t="s">
@@ -14501,19 +14679,19 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="105" t="s">
+      <c r="A12" s="119" t="s">
         <v>1278</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="96"/>
-      <c r="F12" s="96"/>
-      <c r="G12" s="96"/>
-      <c r="H12" s="96"/>
-      <c r="I12" s="96"/>
-      <c r="J12" s="96"/>
-      <c r="K12" s="96"/>
+      <c r="B12" s="110"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="110"/>
+      <c r="K12" s="110"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -14549,49 +14727,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -14630,19 +14808,19 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="99" t="s">
+      <c r="A6" s="113" t="s">
         <v>174</v>
       </c>
-      <c r="B6" s="100"/>
-      <c r="C6" s="100"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="100"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="101"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="114"/>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="114"/>
+      <c r="J6" s="114"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
@@ -14796,19 +14974,19 @@
       <c r="K11" s="18"/>
     </row>
     <row r="12" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="99" t="s">
+      <c r="A12" s="113" t="s">
         <v>184</v>
       </c>
-      <c r="B12" s="100"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="100"/>
-      <c r="E12" s="100"/>
-      <c r="F12" s="100"/>
-      <c r="G12" s="100"/>
-      <c r="H12" s="100"/>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="101"/>
+      <c r="B12" s="114"/>
+      <c r="C12" s="114"/>
+      <c r="D12" s="114"/>
+      <c r="E12" s="114"/>
+      <c r="F12" s="114"/>
+      <c r="G12" s="114"/>
+      <c r="H12" s="114"/>
+      <c r="I12" s="114"/>
+      <c r="J12" s="114"/>
+      <c r="K12" s="115"/>
     </row>
     <row r="13" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
@@ -15347,19 +15525,19 @@
       <c r="K30" s="18"/>
     </row>
     <row r="31" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="99" t="s">
+      <c r="A31" s="113" t="s">
         <v>222</v>
       </c>
-      <c r="B31" s="100"/>
-      <c r="C31" s="100"/>
-      <c r="D31" s="100"/>
-      <c r="E31" s="100"/>
-      <c r="F31" s="100"/>
-      <c r="G31" s="100"/>
-      <c r="H31" s="100"/>
-      <c r="I31" s="100"/>
-      <c r="J31" s="100"/>
-      <c r="K31" s="101"/>
+      <c r="B31" s="114"/>
+      <c r="C31" s="114"/>
+      <c r="D31" s="114"/>
+      <c r="E31" s="114"/>
+      <c r="F31" s="114"/>
+      <c r="G31" s="114"/>
+      <c r="H31" s="114"/>
+      <c r="I31" s="114"/>
+      <c r="J31" s="114"/>
+      <c r="K31" s="115"/>
     </row>
     <row r="32" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
@@ -15567,19 +15745,19 @@
       <c r="K38" s="18"/>
     </row>
     <row r="39" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="99" t="s">
+      <c r="A39" s="113" t="s">
         <v>236</v>
       </c>
-      <c r="B39" s="100"/>
-      <c r="C39" s="100"/>
-      <c r="D39" s="100"/>
-      <c r="E39" s="100"/>
-      <c r="F39" s="100"/>
-      <c r="G39" s="100"/>
-      <c r="H39" s="100"/>
-      <c r="I39" s="100"/>
-      <c r="J39" s="100"/>
-      <c r="K39" s="101"/>
+      <c r="B39" s="114"/>
+      <c r="C39" s="114"/>
+      <c r="D39" s="114"/>
+      <c r="E39" s="114"/>
+      <c r="F39" s="114"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="114"/>
+      <c r="I39" s="114"/>
+      <c r="J39" s="114"/>
+      <c r="K39" s="115"/>
     </row>
     <row r="40" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="17" t="s">
@@ -15729,19 +15907,19 @@
       <c r="K44" s="18"/>
     </row>
     <row r="45" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="99" t="s">
+      <c r="A45" s="113" t="s">
         <v>248</v>
       </c>
-      <c r="B45" s="100"/>
-      <c r="C45" s="100"/>
-      <c r="D45" s="100"/>
-      <c r="E45" s="100"/>
-      <c r="F45" s="100"/>
-      <c r="G45" s="100"/>
-      <c r="H45" s="100"/>
-      <c r="I45" s="100"/>
-      <c r="J45" s="100"/>
-      <c r="K45" s="101"/>
+      <c r="B45" s="114"/>
+      <c r="C45" s="114"/>
+      <c r="D45" s="114"/>
+      <c r="E45" s="114"/>
+      <c r="F45" s="114"/>
+      <c r="G45" s="114"/>
+      <c r="H45" s="114"/>
+      <c r="I45" s="114"/>
+      <c r="J45" s="114"/>
+      <c r="K45" s="115"/>
     </row>
     <row r="46" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="17" t="s">
@@ -15895,19 +16073,19 @@
       <c r="K50" s="18"/>
     </row>
     <row r="51" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="99" t="s">
+      <c r="A51" s="113" t="s">
         <v>259</v>
       </c>
-      <c r="B51" s="100"/>
-      <c r="C51" s="100"/>
-      <c r="D51" s="100"/>
-      <c r="E51" s="100"/>
-      <c r="F51" s="100"/>
-      <c r="G51" s="100"/>
-      <c r="H51" s="100"/>
-      <c r="I51" s="100"/>
-      <c r="J51" s="100"/>
-      <c r="K51" s="101"/>
+      <c r="B51" s="114"/>
+      <c r="C51" s="114"/>
+      <c r="D51" s="114"/>
+      <c r="E51" s="114"/>
+      <c r="F51" s="114"/>
+      <c r="G51" s="114"/>
+      <c r="H51" s="114"/>
+      <c r="I51" s="114"/>
+      <c r="J51" s="114"/>
+      <c r="K51" s="115"/>
     </row>
     <row r="52" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="17" t="s">
@@ -16146,19 +16324,19 @@
       <c r="K59" s="4"/>
     </row>
     <row r="60" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="99" t="s">
+      <c r="A60" s="113" t="s">
         <v>276</v>
       </c>
-      <c r="B60" s="100"/>
-      <c r="C60" s="100"/>
-      <c r="D60" s="100"/>
-      <c r="E60" s="100"/>
-      <c r="F60" s="100"/>
-      <c r="G60" s="100"/>
-      <c r="H60" s="100"/>
-      <c r="I60" s="100"/>
-      <c r="J60" s="100"/>
-      <c r="K60" s="101"/>
+      <c r="B60" s="114"/>
+      <c r="C60" s="114"/>
+      <c r="D60" s="114"/>
+      <c r="E60" s="114"/>
+      <c r="F60" s="114"/>
+      <c r="G60" s="114"/>
+      <c r="H60" s="114"/>
+      <c r="I60" s="114"/>
+      <c r="J60" s="114"/>
+      <c r="K60" s="115"/>
     </row>
     <row r="61" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="21" t="s">
@@ -16422,19 +16600,19 @@
       <c r="K69" s="4"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="99" t="s">
+      <c r="A70" s="113" t="s">
         <v>295</v>
       </c>
-      <c r="B70" s="100"/>
-      <c r="C70" s="100"/>
-      <c r="D70" s="100"/>
-      <c r="E70" s="100"/>
-      <c r="F70" s="100"/>
-      <c r="G70" s="100"/>
-      <c r="H70" s="100"/>
-      <c r="I70" s="100"/>
-      <c r="J70" s="100"/>
-      <c r="K70" s="101"/>
+      <c r="B70" s="114"/>
+      <c r="C70" s="114"/>
+      <c r="D70" s="114"/>
+      <c r="E70" s="114"/>
+      <c r="F70" s="114"/>
+      <c r="G70" s="114"/>
+      <c r="H70" s="114"/>
+      <c r="I70" s="114"/>
+      <c r="J70" s="114"/>
+      <c r="K70" s="115"/>
     </row>
     <row r="71" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="21" t="s">
@@ -16706,19 +16884,19 @@
       <c r="K79" s="4"/>
     </row>
     <row r="80" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="99" t="s">
+      <c r="A80" s="113" t="s">
         <v>314</v>
       </c>
-      <c r="B80" s="100"/>
-      <c r="C80" s="100"/>
-      <c r="D80" s="100"/>
-      <c r="E80" s="100"/>
-      <c r="F80" s="100"/>
-      <c r="G80" s="100"/>
-      <c r="H80" s="100"/>
-      <c r="I80" s="100"/>
-      <c r="J80" s="100"/>
-      <c r="K80" s="101"/>
+      <c r="B80" s="114"/>
+      <c r="C80" s="114"/>
+      <c r="D80" s="114"/>
+      <c r="E80" s="114"/>
+      <c r="F80" s="114"/>
+      <c r="G80" s="114"/>
+      <c r="H80" s="114"/>
+      <c r="I80" s="114"/>
+      <c r="J80" s="114"/>
+      <c r="K80" s="115"/>
     </row>
     <row r="81" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="21" t="s">
@@ -16901,19 +17079,19 @@
       <c r="K86" s="18"/>
     </row>
     <row r="87" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="99" t="s">
+      <c r="A87" s="113" t="s">
         <v>327</v>
       </c>
-      <c r="B87" s="100"/>
-      <c r="C87" s="100"/>
-      <c r="D87" s="100"/>
-      <c r="E87" s="100"/>
-      <c r="F87" s="100"/>
-      <c r="G87" s="100"/>
-      <c r="H87" s="100"/>
-      <c r="I87" s="100"/>
-      <c r="J87" s="100"/>
-      <c r="K87" s="101"/>
+      <c r="B87" s="114"/>
+      <c r="C87" s="114"/>
+      <c r="D87" s="114"/>
+      <c r="E87" s="114"/>
+      <c r="F87" s="114"/>
+      <c r="G87" s="114"/>
+      <c r="H87" s="114"/>
+      <c r="I87" s="114"/>
+      <c r="J87" s="114"/>
+      <c r="K87" s="115"/>
     </row>
     <row r="88" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="17" t="s">
@@ -17187,19 +17365,19 @@
       <c r="K96" s="18"/>
     </row>
     <row r="97" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="99" t="s">
+      <c r="A97" s="113" t="s">
         <v>346</v>
       </c>
-      <c r="B97" s="100"/>
-      <c r="C97" s="100"/>
-      <c r="D97" s="100"/>
-      <c r="E97" s="100"/>
-      <c r="F97" s="100"/>
-      <c r="G97" s="100"/>
-      <c r="H97" s="100"/>
-      <c r="I97" s="100"/>
-      <c r="J97" s="100"/>
-      <c r="K97" s="101"/>
+      <c r="B97" s="114"/>
+      <c r="C97" s="114"/>
+      <c r="D97" s="114"/>
+      <c r="E97" s="114"/>
+      <c r="F97" s="114"/>
+      <c r="G97" s="114"/>
+      <c r="H97" s="114"/>
+      <c r="I97" s="114"/>
+      <c r="J97" s="114"/>
+      <c r="K97" s="115"/>
     </row>
     <row r="98" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="17" t="s">
@@ -17289,19 +17467,19 @@
       <c r="K100" s="18"/>
     </row>
     <row r="101" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="99" t="s">
+      <c r="A101" s="113" t="s">
         <v>222</v>
       </c>
-      <c r="B101" s="100"/>
-      <c r="C101" s="100"/>
-      <c r="D101" s="100"/>
-      <c r="E101" s="100"/>
-      <c r="F101" s="100"/>
-      <c r="G101" s="100"/>
-      <c r="H101" s="100"/>
-      <c r="I101" s="100"/>
-      <c r="J101" s="100"/>
-      <c r="K101" s="101"/>
+      <c r="B101" s="114"/>
+      <c r="C101" s="114"/>
+      <c r="D101" s="114"/>
+      <c r="E101" s="114"/>
+      <c r="F101" s="114"/>
+      <c r="G101" s="114"/>
+      <c r="H101" s="114"/>
+      <c r="I101" s="114"/>
+      <c r="J101" s="114"/>
+      <c r="K101" s="115"/>
     </row>
     <row r="102" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="23" t="s">
@@ -17335,48 +17513,68 @@
       <c r="K102" s="5"/>
     </row>
     <row r="103" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="23" t="s">
+      <c r="A103" s="82" t="s">
         <v>355</v>
       </c>
-      <c r="B103" s="5" t="s">
+      <c r="B103" s="84" t="s">
         <v>222</v>
       </c>
-      <c r="C103" s="24" t="s">
+      <c r="C103" s="83" t="s">
         <v>356</v>
       </c>
-      <c r="D103" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F103" s="5" t="s">
+      <c r="D103" s="84" t="s">
+        <v>97</v>
+      </c>
+      <c r="E103" s="84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F103" s="84" t="s">
         <v>177</v>
       </c>
-      <c r="G103" s="5" t="s">
+      <c r="G103" s="84" t="s">
         <v>178</v>
       </c>
-      <c r="H103" s="5"/>
-      <c r="I103" s="23" t="s">
+      <c r="H103" s="84"/>
+      <c r="I103" s="82" t="s">
         <v>165</v>
       </c>
-      <c r="J103" s="23" t="s">
+      <c r="J103" s="82" t="s">
         <v>166</v>
       </c>
-      <c r="K103" s="5"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A104" s="38"/>
-      <c r="B104" s="38"/>
-      <c r="C104" s="38"/>
-      <c r="D104" s="38"/>
-      <c r="E104" s="38"/>
-      <c r="F104" s="38"/>
-      <c r="G104" s="38"/>
-      <c r="H104" s="38"/>
-      <c r="I104" s="38"/>
-      <c r="J104" s="38"/>
-      <c r="K104" s="38"/>
+      <c r="K103" s="84"/>
+    </row>
+    <row r="104" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="133" t="s">
+        <v>1556</v>
+      </c>
+      <c r="B104" s="131" t="s">
+        <v>327</v>
+      </c>
+      <c r="C104" s="132" t="s">
+        <v>1557</v>
+      </c>
+      <c r="D104" s="85" t="s">
+        <v>97</v>
+      </c>
+      <c r="E104" s="85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F104" s="85" t="s">
+        <v>177</v>
+      </c>
+      <c r="G104" s="85" t="s">
+        <v>178</v>
+      </c>
+      <c r="H104" s="85" t="s">
+        <v>1558</v>
+      </c>
+      <c r="I104" s="133" t="s">
+        <v>1453</v>
+      </c>
+      <c r="J104" s="133" t="s">
+        <v>166</v>
+      </c>
+      <c r="K104" s="124"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="38"/>
@@ -17406,13 +17604,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A101:K101"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A31:K31"/>
-    <mergeCell ref="A97:K97"/>
-    <mergeCell ref="A87:K87"/>
-    <mergeCell ref="A60:K60"/>
-    <mergeCell ref="A39:K39"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A45:K45"/>
@@ -17421,6 +17612,13 @@
     <mergeCell ref="A6:K6"/>
     <mergeCell ref="A70:K70"/>
     <mergeCell ref="A51:K51"/>
+    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A97:K97"/>
+    <mergeCell ref="A87:K87"/>
+    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="A39:K39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17448,49 +17646,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>358</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>359</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -18238,38 +18436,38 @@
       <c r="J29" s="74" t="s">
         <v>166</v>
       </c>
-      <c r="K29" s="93"/>
+      <c r="K29" s="90"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="91" t="s">
+      <c r="A30" s="88" t="s">
         <v>1471</v>
       </c>
-      <c r="B30" s="91" t="s">
+      <c r="B30" s="88" t="s">
         <v>361</v>
       </c>
-      <c r="C30" s="90" t="s">
+      <c r="C30" s="87" t="s">
         <v>1472</v>
       </c>
       <c r="D30" s="80" t="s">
         <v>97</v>
       </c>
-      <c r="E30" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F30" s="91" t="s">
+      <c r="E30" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="88" t="s">
         <v>177</v>
       </c>
-      <c r="G30" s="91" t="s">
+      <c r="G30" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H30" s="91"/>
-      <c r="I30" s="91" t="s">
+      <c r="H30" s="88"/>
+      <c r="I30" s="88" t="s">
         <v>1450</v>
       </c>
-      <c r="J30" s="91" t="s">
+      <c r="J30" s="88" t="s">
         <v>166</v>
       </c>
-      <c r="K30" s="94" t="s">
+      <c r="K30" s="91" t="s">
         <v>1473</v>
       </c>
     </row>
@@ -18336,49 +18534,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>415</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>416</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>417</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -18872,7 +19070,7 @@
   <sheetPr>
     <tabColor rgb="FF2C5F8A"/>
   </sheetPr>
-  <dimension ref="A1:M95"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -18889,19 +19087,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>1479</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
       <c r="L1" t="s">
         <v>1288</v>
       </c>
@@ -18910,34 +19108,34 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>458</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>459</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:13" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:13" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -19721,19 +19919,19 @@
       <c r="K30" s="43"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="114" t="s">
+      <c r="A31" s="106" t="s">
         <v>1289</v>
       </c>
-      <c r="B31" s="115"/>
-      <c r="C31" s="115"/>
-      <c r="D31" s="115"/>
-      <c r="E31" s="115"/>
-      <c r="F31" s="115"/>
-      <c r="G31" s="115"/>
-      <c r="H31" s="115"/>
-      <c r="I31" s="115"/>
-      <c r="J31" s="115"/>
-      <c r="K31" s="116"/>
+      <c r="B31" s="107"/>
+      <c r="C31" s="107"/>
+      <c r="D31" s="107"/>
+      <c r="E31" s="107"/>
+      <c r="F31" s="107"/>
+      <c r="G31" s="107"/>
+      <c r="H31" s="107"/>
+      <c r="I31" s="107"/>
+      <c r="J31" s="107"/>
+      <c r="K31" s="108"/>
     </row>
     <row r="32" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="53" t="s">
@@ -21198,61 +21396,61 @@
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="114" t="s">
+      <c r="A76" s="106" t="s">
         <v>1480</v>
       </c>
-      <c r="B76" s="115"/>
-      <c r="C76" s="115"/>
-      <c r="D76" s="115"/>
-      <c r="E76" s="115"/>
-      <c r="F76" s="115"/>
-      <c r="G76" s="115"/>
-      <c r="H76" s="115"/>
-      <c r="I76" s="115"/>
-      <c r="J76" s="115"/>
-      <c r="K76" s="116"/>
+      <c r="B76" s="107"/>
+      <c r="C76" s="107"/>
+      <c r="D76" s="107"/>
+      <c r="E76" s="107"/>
+      <c r="F76" s="107"/>
+      <c r="G76" s="107"/>
+      <c r="H76" s="107"/>
+      <c r="I76" s="107"/>
+      <c r="J76" s="107"/>
+      <c r="K76" s="108"/>
     </row>
     <row r="77" spans="1:11" ht="58.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="112" t="s">
+      <c r="A77" s="92" t="s">
         <v>1481</v>
       </c>
       <c r="B77" s="60" t="s">
         <v>1480</v>
       </c>
-      <c r="C77" s="117" t="s">
+      <c r="C77" s="94" t="s">
         <v>1482</v>
       </c>
-      <c r="D77" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E77" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F77" s="91" t="s">
+      <c r="D77" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E77" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G77" s="91" t="s">
+      <c r="G77" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H77" s="91"/>
-      <c r="I77" s="91" t="s">
+      <c r="H77" s="88"/>
+      <c r="I77" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J77" s="91" t="s">
+      <c r="J77" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K77" s="94" t="s">
+      <c r="K77" s="91" t="s">
         <v>1483</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A78" s="113" t="s">
+      <c r="A78" s="93" t="s">
         <v>1484</v>
       </c>
       <c r="B78" s="65" t="s">
         <v>1480</v>
       </c>
-      <c r="C78" s="118" t="s">
+      <c r="C78" s="95" t="s">
         <v>1485</v>
       </c>
       <c r="D78" s="74" t="s">
@@ -21279,46 +21477,46 @@
       </c>
     </row>
     <row r="79" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A79" s="112" t="s">
+      <c r="A79" s="92" t="s">
         <v>1487</v>
       </c>
       <c r="B79" s="60" t="s">
         <v>1488</v>
       </c>
-      <c r="C79" s="126" t="s">
+      <c r="C79" s="102" t="s">
         <v>1526</v>
       </c>
-      <c r="D79" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E79" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F79" s="91" t="s">
+      <c r="D79" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E79" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G79" s="91" t="s">
+      <c r="G79" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H79" s="91"/>
-      <c r="I79" s="91" t="s">
+      <c r="H79" s="88"/>
+      <c r="I79" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J79" s="91" t="s">
+      <c r="J79" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K79" s="94" t="s">
+      <c r="K79" s="91" t="s">
         <v>1489</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A80" s="113" t="s">
+      <c r="A80" s="93" t="s">
         <v>1490</v>
       </c>
       <c r="B80" s="65" t="s">
         <v>1491</v>
       </c>
-      <c r="C80" s="118" t="s">
+      <c r="C80" s="95" t="s">
         <v>1492</v>
       </c>
       <c r="D80" s="74" t="s">
@@ -21345,314 +21543,314 @@
       </c>
     </row>
     <row r="81" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A81" s="112" t="s">
+      <c r="A81" s="92" t="s">
         <v>1494</v>
       </c>
       <c r="B81" s="60" t="s">
         <v>1495</v>
       </c>
-      <c r="C81" s="117" t="s">
+      <c r="C81" s="94" t="s">
         <v>1496</v>
       </c>
-      <c r="D81" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E81" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F81" s="91" t="s">
+      <c r="D81" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E81" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G81" s="91" t="s">
+      <c r="G81" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H81" s="91"/>
-      <c r="I81" s="91" t="s">
+      <c r="H81" s="88"/>
+      <c r="I81" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J81" s="91" t="s">
+      <c r="J81" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K81" s="94" t="s">
+      <c r="K81" s="91" t="s">
         <v>1497</v>
       </c>
     </row>
     <row r="82" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A82" s="120" t="s">
+      <c r="A82" s="96" t="s">
         <v>1498</v>
       </c>
-      <c r="B82" s="128" t="s">
+      <c r="B82" s="104" t="s">
         <v>1499</v>
       </c>
-      <c r="C82" s="122" t="s">
+      <c r="C82" s="98" t="s">
         <v>1500</v>
       </c>
-      <c r="D82" s="121" t="s">
-        <v>97</v>
-      </c>
-      <c r="E82" s="121" t="s">
-        <v>8</v>
-      </c>
-      <c r="F82" s="121" t="s">
+      <c r="D82" s="97" t="s">
+        <v>97</v>
+      </c>
+      <c r="E82" s="97" t="s">
+        <v>8</v>
+      </c>
+      <c r="F82" s="97" t="s">
         <v>463</v>
       </c>
-      <c r="G82" s="121" t="s">
+      <c r="G82" s="97" t="s">
         <v>363</v>
       </c>
-      <c r="H82" s="121" t="s">
+      <c r="H82" s="97" t="s">
         <v>117</v>
       </c>
-      <c r="I82" s="121" t="s">
+      <c r="I82" s="97" t="s">
         <v>1171</v>
       </c>
-      <c r="J82" s="121" t="s">
+      <c r="J82" s="97" t="s">
         <v>1282</v>
       </c>
-      <c r="K82" s="123" t="s">
+      <c r="K82" s="99" t="s">
         <v>1501</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A83" s="124" t="s">
+      <c r="A83" s="100" t="s">
         <v>1502</v>
       </c>
-      <c r="B83" s="129" t="s">
+      <c r="B83" s="105" t="s">
         <v>1503</v>
       </c>
-      <c r="C83" s="126" t="s">
+      <c r="C83" s="102" t="s">
         <v>1504</v>
       </c>
-      <c r="D83" s="125" t="s">
-        <v>97</v>
-      </c>
-      <c r="E83" s="125" t="s">
-        <v>8</v>
-      </c>
-      <c r="F83" s="125" t="s">
+      <c r="D83" s="101" t="s">
+        <v>97</v>
+      </c>
+      <c r="E83" s="101" t="s">
+        <v>8</v>
+      </c>
+      <c r="F83" s="101" t="s">
         <v>463</v>
       </c>
-      <c r="G83" s="125" t="s">
+      <c r="G83" s="101" t="s">
         <v>363</v>
       </c>
-      <c r="H83" s="125"/>
-      <c r="I83" s="125" t="s">
+      <c r="H83" s="101"/>
+      <c r="I83" s="101" t="s">
         <v>1171</v>
       </c>
-      <c r="J83" s="125" t="s">
+      <c r="J83" s="101" t="s">
         <v>1282</v>
       </c>
-      <c r="K83" s="127" t="s">
+      <c r="K83" s="103" t="s">
         <v>1505</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="35.4" x14ac:dyDescent="0.3">
-      <c r="A84" s="120" t="s">
+      <c r="A84" s="96" t="s">
         <v>1506</v>
       </c>
-      <c r="B84" s="128" t="s">
+      <c r="B84" s="104" t="s">
         <v>1507</v>
       </c>
-      <c r="C84" s="122" t="s">
+      <c r="C84" s="98" t="s">
         <v>1508</v>
       </c>
-      <c r="D84" s="121" t="s">
-        <v>97</v>
-      </c>
-      <c r="E84" s="121" t="s">
-        <v>8</v>
-      </c>
-      <c r="F84" s="121" t="s">
+      <c r="D84" s="97" t="s">
+        <v>97</v>
+      </c>
+      <c r="E84" s="97" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" s="97" t="s">
         <v>463</v>
       </c>
-      <c r="G84" s="121" t="s">
+      <c r="G84" s="97" t="s">
         <v>363</v>
       </c>
-      <c r="H84" s="121"/>
-      <c r="I84" s="121" t="s">
+      <c r="H84" s="97"/>
+      <c r="I84" s="97" t="s">
         <v>1171</v>
       </c>
-      <c r="J84" s="121" t="s">
+      <c r="J84" s="97" t="s">
         <v>1282</v>
       </c>
-      <c r="K84" s="123" t="s">
+      <c r="K84" s="99" t="s">
         <v>1509</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A85" s="124" t="s">
+      <c r="A85" s="100" t="s">
         <v>1510</v>
       </c>
-      <c r="B85" s="129" t="s">
+      <c r="B85" s="105" t="s">
         <v>1511</v>
       </c>
-      <c r="C85" s="126" t="s">
+      <c r="C85" s="102" t="s">
         <v>1512</v>
       </c>
-      <c r="D85" s="125" t="s">
-        <v>97</v>
-      </c>
-      <c r="E85" s="125" t="s">
-        <v>8</v>
-      </c>
-      <c r="F85" s="125" t="s">
+      <c r="D85" s="101" t="s">
+        <v>97</v>
+      </c>
+      <c r="E85" s="101" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" s="101" t="s">
         <v>463</v>
       </c>
-      <c r="G85" s="125" t="s">
+      <c r="G85" s="101" t="s">
         <v>363</v>
       </c>
-      <c r="H85" s="125" t="s">
+      <c r="H85" s="101" t="s">
         <v>131</v>
       </c>
-      <c r="I85" s="125" t="s">
+      <c r="I85" s="101" t="s">
         <v>1171</v>
       </c>
-      <c r="J85" s="125" t="s">
+      <c r="J85" s="101" t="s">
         <v>1282</v>
       </c>
-      <c r="K85" s="127" t="s">
+      <c r="K85" s="103" t="s">
         <v>1513</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="120" t="s">
+      <c r="A86" s="96" t="s">
         <v>1514</v>
       </c>
-      <c r="B86" s="128" t="s">
+      <c r="B86" s="104" t="s">
         <v>1515</v>
       </c>
-      <c r="C86" s="122" t="s">
+      <c r="C86" s="98" t="s">
         <v>1516</v>
       </c>
-      <c r="D86" s="121" t="s">
+      <c r="D86" s="97" t="s">
         <v>122</v>
       </c>
-      <c r="E86" s="121" t="s">
-        <v>8</v>
-      </c>
-      <c r="F86" s="121" t="s">
+      <c r="E86" s="97" t="s">
+        <v>8</v>
+      </c>
+      <c r="F86" s="97" t="s">
         <v>463</v>
       </c>
-      <c r="G86" s="121" t="s">
+      <c r="G86" s="97" t="s">
         <v>363</v>
       </c>
-      <c r="H86" s="121"/>
-      <c r="I86" s="121" t="s">
+      <c r="H86" s="97"/>
+      <c r="I86" s="97" t="s">
         <v>1171</v>
       </c>
-      <c r="J86" s="121" t="s">
+      <c r="J86" s="97" t="s">
         <v>1282</v>
       </c>
-      <c r="K86" s="123" t="s">
+      <c r="K86" s="99" t="s">
         <v>1517</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="35.4" x14ac:dyDescent="0.3">
-      <c r="A87" s="124" t="s">
+      <c r="A87" s="100" t="s">
         <v>1518</v>
       </c>
-      <c r="B87" s="129" t="s">
+      <c r="B87" s="105" t="s">
         <v>1519</v>
       </c>
-      <c r="C87" s="126" t="s">
+      <c r="C87" s="102" t="s">
         <v>1520</v>
       </c>
-      <c r="D87" s="125" t="s">
+      <c r="D87" s="101" t="s">
         <v>122</v>
       </c>
-      <c r="E87" s="125" t="s">
-        <v>8</v>
-      </c>
-      <c r="F87" s="125" t="s">
+      <c r="E87" s="101" t="s">
+        <v>8</v>
+      </c>
+      <c r="F87" s="101" t="s">
         <v>463</v>
       </c>
-      <c r="G87" s="125" t="s">
+      <c r="G87" s="101" t="s">
         <v>363</v>
       </c>
-      <c r="H87" s="125"/>
-      <c r="I87" s="125" t="s">
+      <c r="H87" s="101"/>
+      <c r="I87" s="101" t="s">
         <v>1171</v>
       </c>
-      <c r="J87" s="125" t="s">
+      <c r="J87" s="101" t="s">
         <v>1282</v>
       </c>
-      <c r="K87" s="127" t="s">
+      <c r="K87" s="103" t="s">
         <v>1521</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="35.4" x14ac:dyDescent="0.3">
-      <c r="A88" s="120" t="s">
+      <c r="A88" s="96" t="s">
         <v>1522</v>
       </c>
-      <c r="B88" s="128" t="s">
+      <c r="B88" s="104" t="s">
         <v>1523</v>
       </c>
-      <c r="C88" s="122" t="s">
+      <c r="C88" s="98" t="s">
         <v>1524</v>
       </c>
-      <c r="D88" s="121" t="s">
+      <c r="D88" s="97" t="s">
         <v>122</v>
       </c>
-      <c r="E88" s="121" t="s">
-        <v>8</v>
-      </c>
-      <c r="F88" s="121" t="s">
+      <c r="E88" s="97" t="s">
+        <v>8</v>
+      </c>
+      <c r="F88" s="97" t="s">
         <v>463</v>
       </c>
-      <c r="G88" s="121" t="s">
+      <c r="G88" s="97" t="s">
         <v>363</v>
       </c>
-      <c r="H88" s="121"/>
-      <c r="I88" s="121" t="s">
+      <c r="H88" s="97"/>
+      <c r="I88" s="97" t="s">
         <v>1171</v>
       </c>
-      <c r="J88" s="121" t="s">
+      <c r="J88" s="97" t="s">
         <v>1282</v>
       </c>
-      <c r="K88" s="123" t="s">
+      <c r="K88" s="99" t="s">
         <v>1525</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A89" s="112" t="s">
+      <c r="A89" s="92" t="s">
         <v>1527</v>
       </c>
       <c r="B89" s="60" t="s">
         <v>1528</v>
       </c>
-      <c r="C89" s="117" t="s">
+      <c r="C89" s="94" t="s">
         <v>1529</v>
       </c>
-      <c r="D89" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E89" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F89" s="91" t="s">
+      <c r="D89" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E89" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F89" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G89" s="91" t="s">
+      <c r="G89" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H89" s="91"/>
-      <c r="I89" s="91" t="s">
+      <c r="H89" s="88"/>
+      <c r="I89" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J89" s="91" t="s">
+      <c r="J89" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K89" s="94" t="s">
+      <c r="K89" s="91" t="s">
         <v>1530</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="92.4" x14ac:dyDescent="0.3">
-      <c r="A90" s="113" t="s">
+      <c r="A90" s="93" t="s">
         <v>1531</v>
       </c>
       <c r="B90" s="65" t="s">
         <v>1532</v>
       </c>
-      <c r="C90" s="118" t="s">
+      <c r="C90" s="95" t="s">
         <v>1533</v>
       </c>
       <c r="D90" s="74" t="s">
@@ -21681,48 +21879,48 @@
       </c>
     </row>
     <row r="91" spans="1:11" ht="69.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A91" s="112" t="s">
+      <c r="A91" s="92" t="s">
         <v>1536</v>
       </c>
       <c r="B91" s="60" t="s">
         <v>1537</v>
       </c>
-      <c r="C91" s="117" t="s">
+      <c r="C91" s="94" t="s">
         <v>1538</v>
       </c>
-      <c r="D91" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E91" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F91" s="91" t="s">
+      <c r="D91" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E91" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F91" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G91" s="91" t="s">
+      <c r="G91" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H91" s="91" t="s">
+      <c r="H91" s="88" t="s">
         <v>117</v>
       </c>
-      <c r="I91" s="91" t="s">
+      <c r="I91" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J91" s="91" t="s">
+      <c r="J91" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K91" s="94" t="s">
+      <c r="K91" s="91" t="s">
         <v>1539</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="69.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A92" s="113" t="s">
+      <c r="A92" s="93" t="s">
         <v>1540</v>
       </c>
       <c r="B92" s="65" t="s">
         <v>1541</v>
       </c>
-      <c r="C92" s="118" t="s">
+      <c r="C92" s="95" t="s">
         <v>1542</v>
       </c>
       <c r="D92" s="74" t="s">
@@ -21749,46 +21947,46 @@
       </c>
     </row>
     <row r="93" spans="1:11" ht="35.4" x14ac:dyDescent="0.3">
-      <c r="A93" s="112" t="s">
+      <c r="A93" s="92" t="s">
         <v>1544</v>
       </c>
       <c r="B93" s="60" t="s">
         <v>1545</v>
       </c>
-      <c r="C93" s="117" t="s">
+      <c r="C93" s="94" t="s">
         <v>1546</v>
       </c>
-      <c r="D93" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="E93" s="91" t="s">
-        <v>8</v>
-      </c>
-      <c r="F93" s="91" t="s">
+      <c r="D93" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E93" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F93" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G93" s="91" t="s">
+      <c r="G93" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H93" s="91"/>
-      <c r="I93" s="91" t="s">
+      <c r="H93" s="88"/>
+      <c r="I93" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J93" s="91" t="s">
+      <c r="J93" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K93" s="94" t="s">
+      <c r="K93" s="91" t="s">
         <v>1547</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="35.4" x14ac:dyDescent="0.3">
-      <c r="A94" s="113" t="s">
+      <c r="A94" s="93" t="s">
         <v>1548</v>
       </c>
       <c r="B94" s="65" t="s">
         <v>1549</v>
       </c>
-      <c r="C94" s="118" t="s">
+      <c r="C94" s="95" t="s">
         <v>1550</v>
       </c>
       <c r="D94" s="74" t="s">
@@ -21815,39 +22013,105 @@
       </c>
     </row>
     <row r="95" spans="1:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A95" s="109" t="s">
+      <c r="A95" s="92" t="s">
         <v>1552</v>
       </c>
-      <c r="B95" s="130" t="s">
+      <c r="B95" s="60" t="s">
         <v>1553</v>
       </c>
-      <c r="C95" s="119" t="s">
+      <c r="C95" s="94" t="s">
         <v>1554</v>
       </c>
-      <c r="D95" s="110" t="s">
-        <v>97</v>
-      </c>
-      <c r="E95" s="110" t="s">
-        <v>8</v>
-      </c>
-      <c r="F95" s="110" t="s">
+      <c r="D95" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="E95" s="88" t="s">
+        <v>8</v>
+      </c>
+      <c r="F95" s="88" t="s">
         <v>463</v>
       </c>
-      <c r="G95" s="110" t="s">
+      <c r="G95" s="88" t="s">
         <v>363</v>
       </c>
-      <c r="H95" s="110" t="s">
+      <c r="H95" s="88" t="s">
         <v>131</v>
       </c>
-      <c r="I95" s="110" t="s">
+      <c r="I95" s="88" t="s">
         <v>1171</v>
       </c>
-      <c r="J95" s="110" t="s">
+      <c r="J95" s="88" t="s">
         <v>1282</v>
       </c>
-      <c r="K95" s="111" t="s">
+      <c r="K95" s="91" t="s">
         <v>1555</v>
       </c>
+    </row>
+    <row r="96" spans="1:11" ht="58.2" x14ac:dyDescent="0.3">
+      <c r="A96" s="125" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B96" s="146" t="s">
+        <v>1559</v>
+      </c>
+      <c r="C96" s="147" t="s">
+        <v>1560</v>
+      </c>
+      <c r="D96" s="123" t="s">
+        <v>97</v>
+      </c>
+      <c r="E96" s="123" t="s">
+        <v>7</v>
+      </c>
+      <c r="F96" s="123" t="s">
+        <v>463</v>
+      </c>
+      <c r="G96" s="123" t="s">
+        <v>363</v>
+      </c>
+      <c r="H96" s="123" t="s">
+        <v>1558</v>
+      </c>
+      <c r="I96" s="139" t="s">
+        <v>1453</v>
+      </c>
+      <c r="J96" s="139" t="s">
+        <v>166</v>
+      </c>
+      <c r="K96" s="148"/>
+    </row>
+    <row r="97" spans="1:11" ht="69.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A97" s="133" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B97" s="134" t="s">
+        <v>1561</v>
+      </c>
+      <c r="C97" s="135" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D97" s="136" t="s">
+        <v>97</v>
+      </c>
+      <c r="E97" s="136" t="s">
+        <v>7</v>
+      </c>
+      <c r="F97" s="136" t="s">
+        <v>463</v>
+      </c>
+      <c r="G97" s="136" t="s">
+        <v>363</v>
+      </c>
+      <c r="H97" s="136" t="s">
+        <v>131</v>
+      </c>
+      <c r="I97" s="133" t="s">
+        <v>1453</v>
+      </c>
+      <c r="J97" s="133" t="s">
+        <v>166</v>
+      </c>
+      <c r="K97" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -21883,49 +22147,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>512</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>513</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>514</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -22560,49 +22824,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>563</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>564</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>565</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -23001,49 +23265,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="111" t="s">
         <v>597</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
     </row>
     <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="109" t="s">
         <v>598</v>
       </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="96"/>
-      <c r="J2" s="96"/>
-      <c r="K2" s="96"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
     </row>
     <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="A3" s="112" t="s">
         <v>599</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="110"/>
+      <c r="I3" s="110"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="110"/>
     </row>
     <row r="4" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>